<commit_message>
add latest client version name
</commit_message>
<xml_diff>
--- a/services/ami/ami/ami_weekly_status_report/per_project/Sweetfoot2/Sweetfoot2_wsr_template_v03.xlsx
+++ b/services/ami/ami/ami_weekly_status_report/per_project/Sweetfoot2/Sweetfoot2_wsr_template_v03.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="1" state="visible" r:id="rId2"/>
@@ -329,7 +329,7 @@
     <t xml:space="preserve">{sg_status_list}</t>
   </si>
   <si>
-    <t xml:space="preserve">v001</t>
+    <t xml:space="preserve">{latest_client_version_sent_version_suffix}</t>
   </si>
   <si>
     <t xml:space="preserve">{layout___sg_blocking_date}</t>
@@ -824,7 +824,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -955,10 +955,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2508,7 +2504,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:W1048576"/>
-  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.18359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.4"/>
@@ -2518,7 +2514,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="36.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="25.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="25.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14.09"/>
@@ -2619,7 +2615,7 @@
       <c r="H3" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="33" t="s">
+      <c r="I3" s="31" t="s">
         <v>61</v>
       </c>
       <c r="J3" s="31" t="s">
@@ -2628,7 +2624,7 @@
       <c r="K3" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="L3" s="34" t="s">
+      <c r="L3" s="33" t="s">
         <v>64</v>
       </c>
       <c r="M3" s="31" t="s">
@@ -2717,15 +2713,15 @@
       <c r="B7" s="31"/>
       <c r="C7" s="31"/>
       <c r="D7" s="31"/>
-      <c r="E7" s="35"/>
+      <c r="E7" s="34"/>
       <c r="F7" s="31"/>
       <c r="G7" s="31"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="35"/>
-      <c r="L7" s="35"/>
-      <c r="M7" s="35"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="34"/>
       <c r="N7" s="31"/>
       <c r="O7" s="31"/>
       <c r="P7" s="31"/>
@@ -2739,15 +2735,15 @@
       <c r="B8" s="31"/>
       <c r="C8" s="31"/>
       <c r="D8" s="31"/>
-      <c r="E8" s="35"/>
+      <c r="E8" s="34"/>
       <c r="F8" s="31"/>
       <c r="G8" s="31"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="35"/>
-      <c r="L8" s="35"/>
-      <c r="M8" s="35"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="34"/>
+      <c r="M8" s="34"/>
       <c r="N8" s="31"/>
       <c r="O8" s="31"/>
       <c r="P8" s="31"/>
@@ -2760,15 +2756,15 @@
       <c r="B9" s="31"/>
       <c r="C9" s="31"/>
       <c r="D9" s="31"/>
-      <c r="E9" s="35"/>
+      <c r="E9" s="34"/>
       <c r="F9" s="31"/>
       <c r="G9" s="31"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="35"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="34"/>
+      <c r="K9" s="34"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="34"/>
       <c r="N9" s="31"/>
       <c r="O9" s="31"/>
       <c r="P9" s="31"/>
@@ -2778,18 +2774,18 @@
       <c r="T9" s="32"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="36"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="38"/>
-      <c r="K10" s="35"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="35"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="38"/>
+      <c r="M10" s="34"/>
       <c r="N10" s="31"/>
       <c r="O10" s="31"/>
       <c r="P10" s="31"/>
@@ -2802,15 +2798,15 @@
       <c r="B11" s="31"/>
       <c r="C11" s="31"/>
       <c r="D11" s="31"/>
-      <c r="E11" s="35"/>
+      <c r="E11" s="34"/>
       <c r="F11" s="31"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="35"/>
-      <c r="L11" s="35"/>
-      <c r="M11" s="35"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="34"/>
       <c r="N11" s="31"/>
       <c r="O11" s="31"/>
       <c r="P11" s="31"/>
@@ -2823,15 +2819,15 @@
       <c r="B12" s="31"/>
       <c r="C12" s="31"/>
       <c r="D12" s="31"/>
-      <c r="E12" s="35"/>
+      <c r="E12" s="34"/>
       <c r="F12" s="31"/>
       <c r="G12" s="31"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
+      <c r="M12" s="34"/>
       <c r="N12" s="31"/>
       <c r="O12" s="31"/>
       <c r="P12" s="31"/>
@@ -2844,15 +2840,15 @@
       <c r="B13" s="31"/>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
-      <c r="E13" s="35"/>
+      <c r="E13" s="34"/>
       <c r="F13" s="31"/>
       <c r="G13" s="31"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="35"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="34"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
+      <c r="M13" s="34"/>
       <c r="N13" s="31"/>
       <c r="O13" s="31"/>
       <c r="P13" s="31"/>
@@ -2865,15 +2861,15 @@
       <c r="B14" s="31"/>
       <c r="C14" s="31"/>
       <c r="D14" s="31"/>
-      <c r="E14" s="35"/>
+      <c r="E14" s="34"/>
       <c r="F14" s="31"/>
       <c r="G14" s="31"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="35"/>
-      <c r="L14" s="35"/>
-      <c r="M14" s="35"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
+      <c r="L14" s="34"/>
+      <c r="M14" s="34"/>
       <c r="N14" s="31"/>
       <c r="O14" s="31"/>
       <c r="P14" s="31"/>
@@ -2886,15 +2882,15 @@
       <c r="B15" s="31"/>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
-      <c r="E15" s="35"/>
+      <c r="E15" s="34"/>
       <c r="F15" s="31"/>
       <c r="G15" s="31"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="35"/>
-      <c r="L15" s="35"/>
-      <c r="M15" s="35"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="34"/>
+      <c r="J15" s="34"/>
+      <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
+      <c r="M15" s="34"/>
       <c r="N15" s="31"/>
       <c r="O15" s="31"/>
       <c r="P15" s="31"/>
@@ -3905,7 +3901,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M1048576"/>
-  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.18359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.31"/>
@@ -3938,7 +3934,7 @@
       <c r="E1" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="39" t="s">
         <v>72</v>
       </c>
       <c r="G1" s="28" t="s">
@@ -3958,10 +3954,10 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="L2" s="35"/>
+      <c r="L2" s="34"/>
       <c r="M2" s="31"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4000,7 +3996,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="40" t="s">
         <v>67</v>
       </c>
       <c r="B4" s="32"/>
@@ -4008,10 +4004,10 @@
       <c r="D4" s="32"/>
       <c r="E4" s="32"/>
       <c r="F4" s="32"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
       <c r="I4" s="31"/>
-      <c r="J4" s="42"/>
+      <c r="J4" s="41"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="32"/>
@@ -4019,10 +4015,10 @@
       <c r="D5" s="32"/>
       <c r="E5" s="32"/>
       <c r="F5" s="32"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="32"/>
@@ -4030,10 +4026,10 @@
       <c r="D6" s="32"/>
       <c r="E6" s="32"/>
       <c r="F6" s="32"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="42"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>